<commit_message>
Number France and GB state mapping rows
</commit_message>
<xml_diff>
--- a/doc/state_mapping.xlsx
+++ b/doc/state_mapping.xlsx
@@ -16227,14 +16227,15 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:C110"/>
+  <dimension ref="A1:D110"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="3" width="17" customWidth="1"/>
+    <col min="4" max="4" width="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>343</v>
       </c>
@@ -16244,8 +16245,13 @@
       <c r="C1" s="2" t="s">
         <v>345</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
         <v>346</v>
       </c>
@@ -16255,8 +16261,11 @@
       <c r="C2" s="4" t="s">
         <v>348</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D2" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
         <v>346</v>
       </c>
@@ -16266,8 +16275,11 @@
       <c r="C3" s="4" t="s">
         <v>350</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D3" s="3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
         <v>346</v>
       </c>
@@ -16277,8 +16289,11 @@
       <c r="C4" s="4" t="s">
         <v>352</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D4" s="3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
         <v>346</v>
       </c>
@@ -16288,8 +16303,11 @@
       <c r="C5" s="4" t="s">
         <v>354</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D5" s="3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
         <v>346</v>
       </c>
@@ -16299,8 +16317,11 @@
       <c r="C6" s="4" t="s">
         <v>356</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D6" s="3">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
         <v>346</v>
       </c>
@@ -16310,8 +16331,11 @@
       <c r="C7" s="4" t="s">
         <v>358</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D7" s="3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="3" t="s">
         <v>346</v>
       </c>
@@ -16321,8 +16345,11 @@
       <c r="C8" s="4" t="s">
         <v>360</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D8" s="3">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="3" t="s">
         <v>346</v>
       </c>
@@ -16332,8 +16359,11 @@
       <c r="C9" s="4" t="s">
         <v>362</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D9" s="3">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="3" t="s">
         <v>346</v>
       </c>
@@ -16343,8 +16373,11 @@
       <c r="C10" s="4" t="s">
         <v>364</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D10" s="3">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="3" t="s">
         <v>346</v>
       </c>
@@ -16354,8 +16387,11 @@
       <c r="C11" s="4" t="s">
         <v>365</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D11" s="3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="3" t="s">
         <v>346</v>
       </c>
@@ -16365,8 +16401,11 @@
       <c r="C12" s="4" t="s">
         <v>366</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D12" s="3">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="3" t="s">
         <v>346</v>
       </c>
@@ -16376,8 +16415,11 @@
       <c r="C13" s="4" t="s">
         <v>367</v>
       </c>
-    </row>
-    <row r="14" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D13" s="3">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="3" t="s">
         <v>346</v>
       </c>
@@ -16387,8 +16429,11 @@
       <c r="C14" s="4" t="s">
         <v>368</v>
       </c>
-    </row>
-    <row r="15" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D14" s="3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="3" t="s">
         <v>346</v>
       </c>
@@ -16398,8 +16443,11 @@
       <c r="C15" s="4" t="s">
         <v>369</v>
       </c>
-    </row>
-    <row r="16" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D15" s="3">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="3" t="s">
         <v>346</v>
       </c>
@@ -16409,8 +16457,11 @@
       <c r="C16" s="4" t="s">
         <v>370</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D16" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="3" t="s">
         <v>346</v>
       </c>
@@ -16420,8 +16471,11 @@
       <c r="C17" s="4" t="s">
         <v>371</v>
       </c>
-    </row>
-    <row r="18" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D17" s="3">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="3" t="s">
         <v>346</v>
       </c>
@@ -16431,8 +16485,11 @@
       <c r="C18" s="4" t="s">
         <v>372</v>
       </c>
-    </row>
-    <row r="19" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D18" s="3">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="3" t="s">
         <v>346</v>
       </c>
@@ -16442,8 +16499,11 @@
       <c r="C19" s="4" t="s">
         <v>373</v>
       </c>
-    </row>
-    <row r="20" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D19" s="3">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="3" t="s">
         <v>346</v>
       </c>
@@ -16453,8 +16513,11 @@
       <c r="C20" s="4" t="s">
         <v>374</v>
       </c>
-    </row>
-    <row r="21" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D20" s="3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="3" t="s">
         <v>346</v>
       </c>
@@ -16464,8 +16527,11 @@
       <c r="C21" s="4" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="22" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D21" s="3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="3" t="s">
         <v>346</v>
       </c>
@@ -16475,8 +16541,11 @@
       <c r="C22" s="4" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="23" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D22" s="3">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="3" t="s">
         <v>346</v>
       </c>
@@ -16486,8 +16555,11 @@
       <c r="C23" s="4" t="s">
         <v>375</v>
       </c>
-    </row>
-    <row r="24" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D23" s="3">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="3" t="s">
         <v>346</v>
       </c>
@@ -16497,8 +16569,11 @@
       <c r="C24" s="4" t="s">
         <v>376</v>
       </c>
-    </row>
-    <row r="25" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D24" s="3">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="3" t="s">
         <v>346</v>
       </c>
@@ -16508,8 +16583,11 @@
       <c r="C25" s="4" t="s">
         <v>377</v>
       </c>
-    </row>
-    <row r="26" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D25" s="3">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="3" t="s">
         <v>346</v>
       </c>
@@ -16519,8 +16597,11 @@
       <c r="C26" s="4" t="s">
         <v>378</v>
       </c>
-    </row>
-    <row r="27" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D26" s="3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="3" t="s">
         <v>346</v>
       </c>
@@ -16530,8 +16611,11 @@
       <c r="C27" s="4" t="s">
         <v>379</v>
       </c>
-    </row>
-    <row r="28" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D27" s="3">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="3" t="s">
         <v>346</v>
       </c>
@@ -16541,8 +16625,11 @@
       <c r="C28" s="4" t="s">
         <v>380</v>
       </c>
-    </row>
-    <row r="29" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D28" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="3" t="s">
         <v>346</v>
       </c>
@@ -16552,8 +16639,11 @@
       <c r="C29" s="4" t="s">
         <v>381</v>
       </c>
-    </row>
-    <row r="30" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D29" s="3">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="3" t="s">
         <v>346</v>
       </c>
@@ -16563,8 +16653,11 @@
       <c r="C30" s="4" t="s">
         <v>382</v>
       </c>
-    </row>
-    <row r="31" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D30" s="3">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="3" t="s">
         <v>346</v>
       </c>
@@ -16574,8 +16667,11 @@
       <c r="C31" s="4" t="s">
         <v>383</v>
       </c>
-    </row>
-    <row r="32" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D31" s="3">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="3" t="s">
         <v>346</v>
       </c>
@@ -16585,8 +16681,11 @@
       <c r="C32" s="4" t="s">
         <v>384</v>
       </c>
-    </row>
-    <row r="33" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D32" s="3">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="3" t="s">
         <v>346</v>
       </c>
@@ -16596,8 +16695,11 @@
       <c r="C33" s="4" t="s">
         <v>385</v>
       </c>
-    </row>
-    <row r="34" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D33" s="3">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="3" t="s">
         <v>346</v>
       </c>
@@ -16607,8 +16709,11 @@
       <c r="C34" s="4" t="s">
         <v>386</v>
       </c>
-    </row>
-    <row r="35" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D34" s="3">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="3" t="s">
         <v>346</v>
       </c>
@@ -16618,8 +16723,11 @@
       <c r="C35" s="4" t="s">
         <v>387</v>
       </c>
-    </row>
-    <row r="36" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D35" s="3">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="3" t="s">
         <v>346</v>
       </c>
@@ -16629,8 +16737,11 @@
       <c r="C36" s="4" t="s">
         <v>388</v>
       </c>
-    </row>
-    <row r="37" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D36" s="3">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="3" t="s">
         <v>346</v>
       </c>
@@ -16640,8 +16751,11 @@
       <c r="C37" s="4" t="s">
         <v>389</v>
       </c>
-    </row>
-    <row r="38" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D37" s="3">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="3" t="s">
         <v>346</v>
       </c>
@@ -16651,8 +16765,11 @@
       <c r="C38" s="4" t="s">
         <v>390</v>
       </c>
-    </row>
-    <row r="39" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D38" s="3">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="3" t="s">
         <v>346</v>
       </c>
@@ -16662,8 +16779,11 @@
       <c r="C39" s="4" t="s">
         <v>391</v>
       </c>
-    </row>
-    <row r="40" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D39" s="3">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="3" t="s">
         <v>346</v>
       </c>
@@ -16673,8 +16793,11 @@
       <c r="C40" s="4" t="s">
         <v>392</v>
       </c>
-    </row>
-    <row r="41" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D40" s="3">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="3" t="s">
         <v>346</v>
       </c>
@@ -16684,8 +16807,11 @@
       <c r="C41" s="4" t="s">
         <v>393</v>
       </c>
-    </row>
-    <row r="42" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D41" s="3">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="3" t="s">
         <v>346</v>
       </c>
@@ -16695,8 +16821,11 @@
       <c r="C42" s="4" t="s">
         <v>394</v>
       </c>
-    </row>
-    <row r="43" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D42" s="3">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="3" t="s">
         <v>346</v>
       </c>
@@ -16706,8 +16835,11 @@
       <c r="C43" s="4" t="s">
         <v>395</v>
       </c>
-    </row>
-    <row r="44" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D43" s="3">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="3" t="s">
         <v>346</v>
       </c>
@@ -16717,8 +16849,11 @@
       <c r="C44" s="4" t="s">
         <v>396</v>
       </c>
-    </row>
-    <row r="45" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D44" s="3">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="3" t="s">
         <v>346</v>
       </c>
@@ -16728,8 +16863,11 @@
       <c r="C45" s="4" t="s">
         <v>397</v>
       </c>
-    </row>
-    <row r="46" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D45" s="3">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="3" t="s">
         <v>346</v>
       </c>
@@ -16739,8 +16877,11 @@
       <c r="C46" s="4" t="s">
         <v>398</v>
       </c>
-    </row>
-    <row r="47" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D46" s="3">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="3" t="s">
         <v>346</v>
       </c>
@@ -16750,8 +16891,11 @@
       <c r="C47" s="4" t="s">
         <v>399</v>
       </c>
-    </row>
-    <row r="48" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D47" s="3">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="3" t="s">
         <v>346</v>
       </c>
@@ -16761,8 +16905,11 @@
       <c r="C48" s="4" t="s">
         <v>400</v>
       </c>
-    </row>
-    <row r="49" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D48" s="3">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="3" t="s">
         <v>346</v>
       </c>
@@ -16772,8 +16919,11 @@
       <c r="C49" s="4" t="s">
         <v>401</v>
       </c>
-    </row>
-    <row r="50" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D49" s="3">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="3" t="s">
         <v>346</v>
       </c>
@@ -16783,8 +16933,11 @@
       <c r="C50" s="4" t="s">
         <v>402</v>
       </c>
-    </row>
-    <row r="51" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D50" s="3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="3" t="s">
         <v>346</v>
       </c>
@@ -16794,8 +16947,11 @@
       <c r="C51" s="4" t="s">
         <v>403</v>
       </c>
-    </row>
-    <row r="52" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D51" s="3">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="3" t="s">
         <v>346</v>
       </c>
@@ -16805,8 +16961,11 @@
       <c r="C52" s="4" t="s">
         <v>404</v>
       </c>
-    </row>
-    <row r="53" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D52" s="3">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="3" t="s">
         <v>346</v>
       </c>
@@ -16816,8 +16975,11 @@
       <c r="C53" s="4" t="s">
         <v>405</v>
       </c>
-    </row>
-    <row r="54" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D53" s="3">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="3" t="s">
         <v>346</v>
       </c>
@@ -16827,8 +16989,11 @@
       <c r="C54" s="4" t="s">
         <v>406</v>
       </c>
-    </row>
-    <row r="55" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D54" s="3">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="3" t="s">
         <v>346</v>
       </c>
@@ -16838,8 +17003,11 @@
       <c r="C55" s="4" t="s">
         <v>407</v>
       </c>
-    </row>
-    <row r="56" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D55" s="3">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="3" t="s">
         <v>346</v>
       </c>
@@ -16849,8 +17017,11 @@
       <c r="C56" s="4" t="s">
         <v>408</v>
       </c>
-    </row>
-    <row r="57" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D56" s="3">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="3" t="s">
         <v>346</v>
       </c>
@@ -16860,8 +17031,11 @@
       <c r="C57" s="4" t="s">
         <v>409</v>
       </c>
-    </row>
-    <row r="58" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D57" s="3">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="3" t="s">
         <v>346</v>
       </c>
@@ -16871,8 +17045,11 @@
       <c r="C58" s="4" t="s">
         <v>410</v>
       </c>
-    </row>
-    <row r="59" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D58" s="3">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="3" t="s">
         <v>346</v>
       </c>
@@ -16882,8 +17059,11 @@
       <c r="C59" s="4" t="s">
         <v>411</v>
       </c>
-    </row>
-    <row r="60" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D59" s="3">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="3" t="s">
         <v>346</v>
       </c>
@@ -16893,8 +17073,11 @@
       <c r="C60" s="4" t="s">
         <v>412</v>
       </c>
-    </row>
-    <row r="61" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D60" s="3">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="3" t="s">
         <v>346</v>
       </c>
@@ -16904,8 +17087,11 @@
       <c r="C61" s="4" t="s">
         <v>413</v>
       </c>
-    </row>
-    <row r="62" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D61" s="3">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="3" t="s">
         <v>346</v>
       </c>
@@ -16915,8 +17101,11 @@
       <c r="C62" s="4" t="s">
         <v>414</v>
       </c>
-    </row>
-    <row r="63" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D62" s="3">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="3" t="s">
         <v>346</v>
       </c>
@@ -16926,8 +17115,11 @@
       <c r="C63" s="4" t="s">
         <v>415</v>
       </c>
-    </row>
-    <row r="64" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D63" s="3">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="3" t="s">
         <v>346</v>
       </c>
@@ -16937,8 +17129,11 @@
       <c r="C64" s="4" t="s">
         <v>416</v>
       </c>
-    </row>
-    <row r="65" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D64" s="3">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="3" t="s">
         <v>346</v>
       </c>
@@ -16948,8 +17143,11 @@
       <c r="C65" s="4" t="s">
         <v>417</v>
       </c>
-    </row>
-    <row r="66" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D65" s="3">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" s="3" t="s">
         <v>346</v>
       </c>
@@ -16959,8 +17157,11 @@
       <c r="C66" s="4" t="s">
         <v>418</v>
       </c>
-    </row>
-    <row r="67" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D66" s="3">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A67" s="3" t="s">
         <v>346</v>
       </c>
@@ -16970,8 +17171,11 @@
       <c r="C67" s="4" t="s">
         <v>419</v>
       </c>
-    </row>
-    <row r="68" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D67" s="3">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A68" s="3" t="s">
         <v>346</v>
       </c>
@@ -16981,8 +17185,11 @@
       <c r="C68" s="4" t="s">
         <v>420</v>
       </c>
-    </row>
-    <row r="69" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D68" s="3">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" s="3" t="s">
         <v>346</v>
       </c>
@@ -16992,8 +17199,11 @@
       <c r="C69" s="4" t="s">
         <v>421</v>
       </c>
-    </row>
-    <row r="70" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D69" s="3">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A70" s="3" t="s">
         <v>346</v>
       </c>
@@ -17003,8 +17213,11 @@
       <c r="C70" s="4" t="s">
         <v>422</v>
       </c>
-    </row>
-    <row r="71" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D70" s="3">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A71" s="3" t="s">
         <v>346</v>
       </c>
@@ -17014,8 +17227,11 @@
       <c r="C71" s="4" t="s">
         <v>423</v>
       </c>
-    </row>
-    <row r="72" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D71" s="3">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A72" s="3" t="s">
         <v>346</v>
       </c>
@@ -17025,8 +17241,11 @@
       <c r="C72" s="4" t="s">
         <v>424</v>
       </c>
-    </row>
-    <row r="73" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D72" s="3">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A73" s="3" t="s">
         <v>346</v>
       </c>
@@ -17036,8 +17255,11 @@
       <c r="C73" s="4" t="s">
         <v>425</v>
       </c>
-    </row>
-    <row r="74" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D73" s="3">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A74" s="3" t="s">
         <v>346</v>
       </c>
@@ -17047,8 +17269,11 @@
       <c r="C74" s="4" t="s">
         <v>426</v>
       </c>
-    </row>
-    <row r="75" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D74" s="3">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A75" s="3" t="s">
         <v>346</v>
       </c>
@@ -17058,8 +17283,11 @@
       <c r="C75" s="4" t="s">
         <v>427</v>
       </c>
-    </row>
-    <row r="76" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D75" s="3">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A76" s="3" t="s">
         <v>346</v>
       </c>
@@ -17069,8 +17297,11 @@
       <c r="C76" s="4" t="s">
         <v>428</v>
       </c>
-    </row>
-    <row r="77" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D76" s="3">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A77" s="3" t="s">
         <v>346</v>
       </c>
@@ -17080,8 +17311,11 @@
       <c r="C77" s="4" t="s">
         <v>429</v>
       </c>
-    </row>
-    <row r="78" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D77" s="3">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A78" s="3" t="s">
         <v>346</v>
       </c>
@@ -17091,8 +17325,11 @@
       <c r="C78" s="4" t="s">
         <v>430</v>
       </c>
-    </row>
-    <row r="79" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D78" s="3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A79" s="3" t="s">
         <v>346</v>
       </c>
@@ -17102,8 +17339,11 @@
       <c r="C79" s="4" t="s">
         <v>431</v>
       </c>
-    </row>
-    <row r="80" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D79" s="3">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A80" s="3" t="s">
         <v>346</v>
       </c>
@@ -17113,8 +17353,11 @@
       <c r="C80" s="4" t="s">
         <v>432</v>
       </c>
-    </row>
-    <row r="81" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D80" s="3">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A81" s="3" t="s">
         <v>346</v>
       </c>
@@ -17124,8 +17367,11 @@
       <c r="C81" s="4" t="s">
         <v>433</v>
       </c>
-    </row>
-    <row r="82" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D81" s="3">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A82" s="3" t="s">
         <v>346</v>
       </c>
@@ -17135,8 +17381,11 @@
       <c r="C82" s="4" t="s">
         <v>434</v>
       </c>
-    </row>
-    <row r="83" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D82" s="3">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A83" s="3" t="s">
         <v>346</v>
       </c>
@@ -17146,8 +17395,11 @@
       <c r="C83" s="4" t="s">
         <v>435</v>
       </c>
-    </row>
-    <row r="84" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D83" s="3">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A84" s="3" t="s">
         <v>346</v>
       </c>
@@ -17157,8 +17409,11 @@
       <c r="C84" s="4" t="s">
         <v>436</v>
       </c>
-    </row>
-    <row r="85" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D84" s="3">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A85" s="3" t="s">
         <v>346</v>
       </c>
@@ -17168,8 +17423,11 @@
       <c r="C85" s="4" t="s">
         <v>437</v>
       </c>
-    </row>
-    <row r="86" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D85" s="3">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A86" s="3" t="s">
         <v>346</v>
       </c>
@@ -17179,8 +17437,11 @@
       <c r="C86" s="4" t="s">
         <v>438</v>
       </c>
-    </row>
-    <row r="87" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D86" s="3">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A87" s="3" t="s">
         <v>346</v>
       </c>
@@ -17190,8 +17451,11 @@
       <c r="C87" s="4" t="s">
         <v>439</v>
       </c>
-    </row>
-    <row r="88" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D87" s="3">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A88" s="3" t="s">
         <v>346</v>
       </c>
@@ -17201,8 +17465,11 @@
       <c r="C88" s="4" t="s">
         <v>440</v>
       </c>
-    </row>
-    <row r="89" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D88" s="3">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A89" s="3" t="s">
         <v>346</v>
       </c>
@@ -17212,8 +17479,11 @@
       <c r="C89" s="4" t="s">
         <v>441</v>
       </c>
-    </row>
-    <row r="90" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D89" s="3">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A90" s="3" t="s">
         <v>346</v>
       </c>
@@ -17223,8 +17493,11 @@
       <c r="C90" s="4" t="s">
         <v>442</v>
       </c>
-    </row>
-    <row r="91" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D90" s="3">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A91" s="3" t="s">
         <v>346</v>
       </c>
@@ -17234,8 +17507,11 @@
       <c r="C91" s="4" t="s">
         <v>443</v>
       </c>
-    </row>
-    <row r="92" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D91" s="3">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A92" s="3" t="s">
         <v>346</v>
       </c>
@@ -17245,8 +17521,11 @@
       <c r="C92" s="4" t="s">
         <v>444</v>
       </c>
-    </row>
-    <row r="93" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D92" s="3">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A93" s="3" t="s">
         <v>346</v>
       </c>
@@ -17256,8 +17535,11 @@
       <c r="C93" s="4" t="s">
         <v>445</v>
       </c>
-    </row>
-    <row r="94" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D93" s="3">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="94" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A94" s="3" t="s">
         <v>346</v>
       </c>
@@ -17267,8 +17549,11 @@
       <c r="C94" s="4" t="s">
         <v>446</v>
       </c>
-    </row>
-    <row r="95" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D94" s="3">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="95" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A95" s="3" t="s">
         <v>346</v>
       </c>
@@ -17278,8 +17563,11 @@
       <c r="C95" s="4" t="s">
         <v>447</v>
       </c>
-    </row>
-    <row r="96" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D95" s="3">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="96" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A96" s="3" t="s">
         <v>346</v>
       </c>
@@ -17289,8 +17577,11 @@
       <c r="C96" s="4" t="s">
         <v>448</v>
       </c>
-    </row>
-    <row r="97" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D96" s="3">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="97" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A97" s="3" t="s">
         <v>346</v>
       </c>
@@ -17300,8 +17591,11 @@
       <c r="C97" s="4" t="s">
         <v>449</v>
       </c>
-    </row>
-    <row r="98" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D97" s="3">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="98" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A98" s="3" t="s">
         <v>346</v>
       </c>
@@ -17311,8 +17605,11 @@
       <c r="C98" s="4" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="99" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D98" s="3">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="99" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A99" s="3" t="s">
         <v>346</v>
       </c>
@@ -17322,8 +17619,11 @@
       <c r="C99" s="4" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="100" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D99" s="3">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="100" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A100" s="3" t="s">
         <v>346</v>
       </c>
@@ -17333,8 +17633,11 @@
       <c r="C100" s="4" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="101" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D100" s="3">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="101" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A101" s="3" t="s">
         <v>346</v>
       </c>
@@ -17344,8 +17647,11 @@
       <c r="C101" s="4" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="102" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D101" s="3">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="102" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A102" s="3" t="s">
         <v>346</v>
       </c>
@@ -17355,8 +17661,11 @@
       <c r="C102" s="4" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="103" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D102" s="3">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="103" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A103" s="3" t="s">
         <v>346</v>
       </c>
@@ -17366,8 +17675,11 @@
       <c r="C103" s="4" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="104" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D103" s="3">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="104" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A104" s="3" t="s">
         <v>346</v>
       </c>
@@ -17375,8 +17687,11 @@
       <c r="C104" s="4" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="105" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D104" s="3">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="105" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A105" s="3" t="s">
         <v>346</v>
       </c>
@@ -17384,8 +17699,11 @@
       <c r="C105" s="4" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="106" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D105" s="3">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="106" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A106" s="3" t="s">
         <v>346</v>
       </c>
@@ -17393,8 +17711,11 @@
       <c r="C106" s="4" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="107" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D106" s="3">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="107" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A107" s="3" t="s">
         <v>346</v>
       </c>
@@ -17402,8 +17723,11 @@
       <c r="C107" s="4" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="108" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D107" s="3">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="108" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A108" s="3" t="s">
         <v>346</v>
       </c>
@@ -17411,8 +17735,11 @@
       <c r="C108" s="4" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="109" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D108" s="3">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="109" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A109" s="3" t="s">
         <v>346</v>
       </c>
@@ -17420,14 +17747,20 @@
       <c r="C109" s="4" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="110" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D109" s="3">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="110" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A110" s="3" t="s">
         <v>346</v>
       </c>
       <c r="B110" s="5"/>
       <c r="C110" s="4" t="s">
         <v>41</v>
+      </c>
+      <c r="D110" s="3">
+        <v>109</v>
       </c>
     </row>
   </sheetData>
@@ -17439,14 +17772,15 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:C222"/>
+  <dimension ref="A1:D222"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="3" width="17" customWidth="1"/>
+    <col min="4" max="4" width="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>343</v>
       </c>
@@ -17456,8 +17790,13 @@
       <c r="C1" s="2" t="s">
         <v>345</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -17473,8 +17812,11 @@
           <t>BKM</t>
         </is>
       </c>
-    </row>
-    <row r="3" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D2" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -17490,8 +17832,11 @@
           <t>CAM</t>
         </is>
       </c>
-    </row>
-    <row r="4" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D3" s="3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -17507,8 +17852,11 @@
           <t>CMA</t>
         </is>
       </c>
-    </row>
-    <row r="5" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D4" s="3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -17524,8 +17872,11 @@
           <t>DBY</t>
         </is>
       </c>
-    </row>
-    <row r="6" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D5" s="3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -17541,8 +17892,11 @@
           <t>DEV</t>
         </is>
       </c>
-    </row>
-    <row r="7" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D6" s="3">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -17558,8 +17912,11 @@
           <t>DOR</t>
         </is>
       </c>
-    </row>
-    <row r="8" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D7" s="3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -17575,8 +17932,11 @@
           <t>ESX</t>
         </is>
       </c>
-    </row>
-    <row r="9" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D8" s="3">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -17592,8 +17952,11 @@
           <t>ESS</t>
         </is>
       </c>
-    </row>
-    <row r="10" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D9" s="3">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -17609,8 +17972,11 @@
           <t>GLS</t>
         </is>
       </c>
-    </row>
-    <row r="11" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D10" s="3">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -17626,8 +17992,11 @@
           <t>HAM</t>
         </is>
       </c>
-    </row>
-    <row r="12" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D11" s="3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -17643,8 +18012,11 @@
           <t>HRT</t>
         </is>
       </c>
-    </row>
-    <row r="13" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D12" s="3">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -17660,8 +18032,11 @@
           <t>KEN</t>
         </is>
       </c>
-    </row>
-    <row r="14" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D13" s="3">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -17677,8 +18052,11 @@
           <t>LAN</t>
         </is>
       </c>
-    </row>
-    <row r="15" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D14" s="3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -17694,8 +18072,11 @@
           <t>LEC</t>
         </is>
       </c>
-    </row>
-    <row r="16" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D15" s="3">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -17711,8 +18092,11 @@
           <t>LIN</t>
         </is>
       </c>
-    </row>
-    <row r="17" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D16" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -17728,8 +18112,11 @@
           <t>NFK</t>
         </is>
       </c>
-    </row>
-    <row r="18" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D17" s="3">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -17745,8 +18132,11 @@
           <t>NYK</t>
         </is>
       </c>
-    </row>
-    <row r="19" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D18" s="3">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -17762,8 +18152,11 @@
           <t>NTH</t>
         </is>
       </c>
-    </row>
-    <row r="20" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D19" s="3">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -17779,8 +18172,11 @@
           <t>NTT</t>
         </is>
       </c>
-    </row>
-    <row r="21" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D20" s="3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -17796,8 +18192,11 @@
           <t>OXF</t>
         </is>
       </c>
-    </row>
-    <row r="22" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D21" s="3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -17813,8 +18212,11 @@
           <t>SOM</t>
         </is>
       </c>
-    </row>
-    <row r="23" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D22" s="3">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -17830,8 +18232,11 @@
           <t>STS</t>
         </is>
       </c>
-    </row>
-    <row r="24" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D23" s="3">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -17847,8 +18252,11 @@
           <t>SFK</t>
         </is>
       </c>
-    </row>
-    <row r="25" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D24" s="3">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -17864,8 +18272,11 @@
           <t>SRY</t>
         </is>
       </c>
-    </row>
-    <row r="26" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D25" s="3">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -17881,8 +18292,11 @@
           <t>WAR</t>
         </is>
       </c>
-    </row>
-    <row r="27" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D26" s="3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -17898,8 +18312,11 @@
           <t>WSX</t>
         </is>
       </c>
-    </row>
-    <row r="28" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D27" s="3">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -17915,8 +18332,11 @@
           <t>WOR</t>
         </is>
       </c>
-    </row>
-    <row r="29" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D28" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -17932,8 +18352,11 @@
           <t>BDG</t>
         </is>
       </c>
-    </row>
-    <row r="30" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D29" s="3">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -17949,8 +18372,11 @@
           <t>BNE</t>
         </is>
       </c>
-    </row>
-    <row r="31" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D30" s="3">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -17966,8 +18392,11 @@
           <t>BEX</t>
         </is>
       </c>
-    </row>
-    <row r="32" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D31" s="3">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -17983,8 +18412,11 @@
           <t>BEN</t>
         </is>
       </c>
-    </row>
-    <row r="33" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D32" s="3">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -18000,8 +18432,11 @@
           <t>BRY</t>
         </is>
       </c>
-    </row>
-    <row r="34" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D33" s="3">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -18017,8 +18452,11 @@
           <t>CMD</t>
         </is>
       </c>
-    </row>
-    <row r="35" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D34" s="3">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -18034,8 +18472,11 @@
           <t>CRY</t>
         </is>
       </c>
-    </row>
-    <row r="36" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D35" s="3">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -18051,8 +18492,11 @@
           <t>EAL</t>
         </is>
       </c>
-    </row>
-    <row r="37" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D36" s="3">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -18068,8 +18512,11 @@
           <t>ENF</t>
         </is>
       </c>
-    </row>
-    <row r="38" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D37" s="3">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -18085,8 +18532,11 @@
           <t>GRE</t>
         </is>
       </c>
-    </row>
-    <row r="39" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D38" s="3">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -18102,8 +18552,11 @@
           <t>HCK</t>
         </is>
       </c>
-    </row>
-    <row r="40" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D39" s="3">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -18119,8 +18572,11 @@
           <t>HMF</t>
         </is>
       </c>
-    </row>
-    <row r="41" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D40" s="3">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -18136,8 +18592,11 @@
           <t>HRY</t>
         </is>
       </c>
-    </row>
-    <row r="42" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D41" s="3">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -18153,8 +18612,11 @@
           <t>HRW</t>
         </is>
       </c>
-    </row>
-    <row r="43" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D42" s="3">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -18170,8 +18632,11 @@
           <t>HAV</t>
         </is>
       </c>
-    </row>
-    <row r="44" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D43" s="3">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -18187,8 +18652,11 @@
           <t>HIL</t>
         </is>
       </c>
-    </row>
-    <row r="45" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D44" s="3">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -18204,8 +18672,11 @@
           <t>HNS</t>
         </is>
       </c>
-    </row>
-    <row r="46" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D45" s="3">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -18221,8 +18692,11 @@
           <t>ISL</t>
         </is>
       </c>
-    </row>
-    <row r="47" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D46" s="3">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -18238,8 +18712,11 @@
           <t>KEC</t>
         </is>
       </c>
-    </row>
-    <row r="48" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D47" s="3">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -18255,8 +18732,11 @@
           <t>KTT</t>
         </is>
       </c>
-    </row>
-    <row r="49" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D48" s="3">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -18272,8 +18752,11 @@
           <t>LBH</t>
         </is>
       </c>
-    </row>
-    <row r="50" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D49" s="3">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -18289,8 +18772,11 @@
           <t>LEW</t>
         </is>
       </c>
-    </row>
-    <row r="51" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D50" s="3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -18306,8 +18792,11 @@
           <t>MRT</t>
         </is>
       </c>
-    </row>
-    <row r="52" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D51" s="3">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -18323,8 +18812,11 @@
           <t>NWM</t>
         </is>
       </c>
-    </row>
-    <row r="53" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D52" s="3">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -18340,8 +18832,11 @@
           <t>RDB</t>
         </is>
       </c>
-    </row>
-    <row r="54" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D53" s="3">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -18357,8 +18852,11 @@
           <t>RIC</t>
         </is>
       </c>
-    </row>
-    <row r="55" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D54" s="3">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -18374,8 +18872,11 @@
           <t>SWK</t>
         </is>
       </c>
-    </row>
-    <row r="56" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D55" s="3">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -18391,8 +18892,11 @@
           <t>STN</t>
         </is>
       </c>
-    </row>
-    <row r="57" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D56" s="3">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -18408,8 +18912,11 @@
           <t>TWH</t>
         </is>
       </c>
-    </row>
-    <row r="58" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D57" s="3">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -18425,8 +18932,11 @@
           <t>WFT</t>
         </is>
       </c>
-    </row>
-    <row r="59" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D58" s="3">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -18442,8 +18952,11 @@
           <t>WND</t>
         </is>
       </c>
-    </row>
-    <row r="60" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D59" s="3">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -18459,8 +18972,11 @@
           <t>WSM</t>
         </is>
       </c>
-    </row>
-    <row r="61" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D60" s="3">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -18476,8 +18992,11 @@
           <t>BNS</t>
         </is>
       </c>
-    </row>
-    <row r="62" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D61" s="3">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -18493,8 +19012,11 @@
           <t>BIR</t>
         </is>
       </c>
-    </row>
-    <row r="63" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D62" s="3">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -18510,8 +19032,11 @@
           <t>BOL</t>
         </is>
       </c>
-    </row>
-    <row r="64" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D63" s="3">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -18527,8 +19052,11 @@
           <t>BRD</t>
         </is>
       </c>
-    </row>
-    <row r="65" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D64" s="3">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -18544,8 +19072,11 @@
           <t>BUR</t>
         </is>
       </c>
-    </row>
-    <row r="66" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D65" s="3">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -18561,8 +19092,11 @@
           <t>CLD</t>
         </is>
       </c>
-    </row>
-    <row r="67" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D66" s="3">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A67" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -18578,8 +19112,11 @@
           <t>COV</t>
         </is>
       </c>
-    </row>
-    <row r="68" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D67" s="3">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A68" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -18595,8 +19132,11 @@
           <t>DNC</t>
         </is>
       </c>
-    </row>
-    <row r="69" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D68" s="3">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -18612,8 +19152,11 @@
           <t>DUD</t>
         </is>
       </c>
-    </row>
-    <row r="70" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D69" s="3">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A70" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -18629,8 +19172,11 @@
           <t>GAT</t>
         </is>
       </c>
-    </row>
-    <row r="71" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D70" s="3">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A71" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -18646,8 +19192,11 @@
           <t>KIR</t>
         </is>
       </c>
-    </row>
-    <row r="72" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D71" s="3">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A72" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -18663,8 +19212,11 @@
           <t>KWL</t>
         </is>
       </c>
-    </row>
-    <row r="73" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D72" s="3">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A73" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -18680,8 +19232,11 @@
           <t>LDS</t>
         </is>
       </c>
-    </row>
-    <row r="74" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D73" s="3">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A74" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -18697,8 +19252,11 @@
           <t>LIV</t>
         </is>
       </c>
-    </row>
-    <row r="75" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D74" s="3">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A75" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -18714,8 +19272,11 @@
           <t>MAN</t>
         </is>
       </c>
-    </row>
-    <row r="76" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D75" s="3">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A76" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -18731,8 +19292,11 @@
           <t>NET</t>
         </is>
       </c>
-    </row>
-    <row r="77" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D76" s="3">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A77" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -18748,8 +19312,11 @@
           <t>NTY</t>
         </is>
       </c>
-    </row>
-    <row r="78" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D77" s="3">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A78" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -18765,8 +19332,11 @@
           <t>OLD</t>
         </is>
       </c>
-    </row>
-    <row r="79" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D78" s="3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A79" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -18782,8 +19352,11 @@
           <t>RCH</t>
         </is>
       </c>
-    </row>
-    <row r="80" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D79" s="3">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A80" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -18799,8 +19372,11 @@
           <t>ROT</t>
         </is>
       </c>
-    </row>
-    <row r="81" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D80" s="3">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A81" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -18816,8 +19392,11 @@
           <t>SHN</t>
         </is>
       </c>
-    </row>
-    <row r="82" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D81" s="3">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A82" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -18833,8 +19412,11 @@
           <t>SLF</t>
         </is>
       </c>
-    </row>
-    <row r="83" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D82" s="3">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A83" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -18850,8 +19432,11 @@
           <t>SAW</t>
         </is>
       </c>
-    </row>
-    <row r="84" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D83" s="3">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A84" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -18867,8 +19452,11 @@
           <t>SFT</t>
         </is>
       </c>
-    </row>
-    <row r="85" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D84" s="3">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A85" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -18884,8 +19472,11 @@
           <t>SHF</t>
         </is>
       </c>
-    </row>
-    <row r="86" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D85" s="3">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A86" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -18901,8 +19492,11 @@
           <t>SOL</t>
         </is>
       </c>
-    </row>
-    <row r="87" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D86" s="3">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A87" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -18918,8 +19512,11 @@
           <t>STY</t>
         </is>
       </c>
-    </row>
-    <row r="88" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D87" s="3">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A88" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -18935,8 +19532,11 @@
           <t>SKP</t>
         </is>
       </c>
-    </row>
-    <row r="89" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D88" s="3">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A89" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -18952,8 +19552,11 @@
           <t>SND</t>
         </is>
       </c>
-    </row>
-    <row r="90" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D89" s="3">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A90" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -18969,8 +19572,11 @@
           <t>TAM</t>
         </is>
       </c>
-    </row>
-    <row r="91" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D90" s="3">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A91" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -18986,8 +19592,11 @@
           <t>TRF</t>
         </is>
       </c>
-    </row>
-    <row r="92" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D91" s="3">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A92" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -19003,8 +19612,11 @@
           <t>WKF</t>
         </is>
       </c>
-    </row>
-    <row r="93" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D92" s="3">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A93" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -19020,8 +19632,11 @@
           <t>WLL</t>
         </is>
       </c>
-    </row>
-    <row r="94" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D93" s="3">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="94" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A94" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -19037,8 +19652,11 @@
           <t>WGN</t>
         </is>
       </c>
-    </row>
-    <row r="95" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D94" s="3">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="95" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A95" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -19054,8 +19672,11 @@
           <t>WRL</t>
         </is>
       </c>
-    </row>
-    <row r="96" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D95" s="3">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="96" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A96" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -19071,8 +19692,11 @@
           <t>WLV</t>
         </is>
       </c>
-    </row>
-    <row r="97" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D96" s="3">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="97" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A97" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -19088,8 +19712,11 @@
           <t>BAS</t>
         </is>
       </c>
-    </row>
-    <row r="98" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D97" s="3">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="98" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A98" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -19105,8 +19732,11 @@
           <t>BBD</t>
         </is>
       </c>
-    </row>
-    <row r="99" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D98" s="3">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="99" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A99" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -19122,8 +19752,11 @@
           <t>BDF</t>
         </is>
       </c>
-    </row>
-    <row r="100" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D99" s="3">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="100" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A100" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -19139,8 +19772,11 @@
           <t>BPL</t>
         </is>
       </c>
-    </row>
-    <row r="101" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D100" s="3">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="101" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A101" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -19156,8 +19792,11 @@
           <t>BMH</t>
         </is>
       </c>
-    </row>
-    <row r="102" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D101" s="3">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="102" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A102" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -19173,8 +19812,11 @@
           <t>BRC</t>
         </is>
       </c>
-    </row>
-    <row r="103" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D102" s="3">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="103" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A103" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -19190,8 +19832,11 @@
           <t>BNH</t>
         </is>
       </c>
-    </row>
-    <row r="104" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D103" s="3">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="104" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A104" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -19207,8 +19852,11 @@
           <t>BST</t>
         </is>
       </c>
-    </row>
-    <row r="105" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D104" s="3">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="105" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A105" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -19224,8 +19872,11 @@
           <t>CBF</t>
         </is>
       </c>
-    </row>
-    <row r="106" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D105" s="3">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="106" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A106" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -19241,8 +19892,11 @@
           <t>CHE</t>
         </is>
       </c>
-    </row>
-    <row r="107" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D106" s="3">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="107" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A107" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -19258,8 +19912,11 @@
           <t>CHW</t>
         </is>
       </c>
-    </row>
-    <row r="108" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D107" s="3">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="108" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A108" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -19275,8 +19932,11 @@
           <t>CON</t>
         </is>
       </c>
-    </row>
-    <row r="109" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D108" s="3">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="109" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A109" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -19292,8 +19952,11 @@
           <t>DAL</t>
         </is>
       </c>
-    </row>
-    <row r="110" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D109" s="3">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="110" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A110" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -19309,8 +19972,11 @@
           <t>DER</t>
         </is>
       </c>
-    </row>
-    <row r="111" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D110" s="3">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="111" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A111" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -19326,8 +19992,11 @@
           <t>DUR</t>
         </is>
       </c>
-    </row>
-    <row r="112" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D111" s="3">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="112" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A112" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -19343,8 +20012,11 @@
           <t>ERY</t>
         </is>
       </c>
-    </row>
-    <row r="113" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D112" s="3">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="113" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A113" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -19360,8 +20032,11 @@
           <t>HAL</t>
         </is>
       </c>
-    </row>
-    <row r="114" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D113" s="3">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="114" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A114" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -19377,8 +20052,11 @@
           <t>HPL</t>
         </is>
       </c>
-    </row>
-    <row r="115" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D114" s="3">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="115" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A115" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -19394,8 +20072,11 @@
           <t>HEF</t>
         </is>
       </c>
-    </row>
-    <row r="116" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D115" s="3">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="116" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A116" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -19411,8 +20092,11 @@
           <t>IOW</t>
         </is>
       </c>
-    </row>
-    <row r="117" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D116" s="3">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="117" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A117" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -19428,8 +20112,11 @@
           <t>KHL</t>
         </is>
       </c>
-    </row>
-    <row r="118" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D117" s="3">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="118" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A118" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -19445,8 +20132,11 @@
           <t>LCE</t>
         </is>
       </c>
-    </row>
-    <row r="119" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D118" s="3">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="119" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A119" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -19462,8 +20152,11 @@
           <t>LUT</t>
         </is>
       </c>
-    </row>
-    <row r="120" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D119" s="3">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="120" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A120" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -19479,8 +20172,11 @@
           <t>MDB</t>
         </is>
       </c>
-    </row>
-    <row r="121" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D120" s="3">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="121" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A121" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -19496,8 +20192,11 @@
           <t>MIK</t>
         </is>
       </c>
-    </row>
-    <row r="122" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D121" s="3">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="122" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A122" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -19513,8 +20212,11 @@
           <t>NEL</t>
         </is>
       </c>
-    </row>
-    <row r="123" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D122" s="3">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="123" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A123" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -19530,8 +20232,11 @@
           <t>NLN</t>
         </is>
       </c>
-    </row>
-    <row r="124" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D123" s="3">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="124" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A124" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -19547,8 +20252,11 @@
           <t>NSM</t>
         </is>
       </c>
-    </row>
-    <row r="125" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D124" s="3">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="125" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A125" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -19564,8 +20272,11 @@
           <t>NBL</t>
         </is>
       </c>
-    </row>
-    <row r="126" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D125" s="3">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="126" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A126" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -19581,8 +20292,11 @@
           <t>NGM</t>
         </is>
       </c>
-    </row>
-    <row r="127" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D126" s="3">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="127" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A127" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -19598,8 +20312,11 @@
           <t>PTE</t>
         </is>
       </c>
-    </row>
-    <row r="128" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D127" s="3">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="128" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A128" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -19615,8 +20332,11 @@
           <t>PLY</t>
         </is>
       </c>
-    </row>
-    <row r="129" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D128" s="3">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="129" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A129" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -19632,8 +20352,11 @@
           <t>POL</t>
         </is>
       </c>
-    </row>
-    <row r="130" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D129" s="3">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="130" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A130" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -19649,8 +20372,11 @@
           <t>POR</t>
         </is>
       </c>
-    </row>
-    <row r="131" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D130" s="3">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="131" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A131" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -19666,8 +20392,11 @@
           <t>RDG</t>
         </is>
       </c>
-    </row>
-    <row r="132" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D131" s="3">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="132" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A132" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -19683,8 +20412,11 @@
           <t>RCC</t>
         </is>
       </c>
-    </row>
-    <row r="133" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D132" s="3">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="133" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A133" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -19700,8 +20432,11 @@
           <t>RUT</t>
         </is>
       </c>
-    </row>
-    <row r="134" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D133" s="3">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="134" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A134" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -19717,8 +20452,11 @@
           <t>SHR</t>
         </is>
       </c>
-    </row>
-    <row r="135" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D134" s="3">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="135" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A135" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -19734,8 +20472,11 @@
           <t>SLG</t>
         </is>
       </c>
-    </row>
-    <row r="136" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D135" s="3">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="136" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A136" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -19751,8 +20492,11 @@
           <t>SGC</t>
         </is>
       </c>
-    </row>
-    <row r="137" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D136" s="3">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="137" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A137" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -19768,8 +20512,11 @@
           <t>STH</t>
         </is>
       </c>
-    </row>
-    <row r="138" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D137" s="3">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="138" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A138" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -19785,8 +20532,11 @@
           <t>SOS</t>
         </is>
       </c>
-    </row>
-    <row r="139" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D138" s="3">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="139" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A139" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -19802,8 +20552,11 @@
           <t>STT</t>
         </is>
       </c>
-    </row>
-    <row r="140" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D139" s="3">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="140" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A140" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -19819,8 +20572,11 @@
           <t>STE</t>
         </is>
       </c>
-    </row>
-    <row r="141" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D140" s="3">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="141" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A141" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -19836,8 +20592,11 @@
           <t>SWD</t>
         </is>
       </c>
-    </row>
-    <row r="142" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D141" s="3">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="142" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A142" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -19853,8 +20612,11 @@
           <t>TFW</t>
         </is>
       </c>
-    </row>
-    <row r="143" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D142" s="3">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="143" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A143" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -19870,8 +20632,11 @@
           <t>THR</t>
         </is>
       </c>
-    </row>
-    <row r="144" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D143" s="3">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="144" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A144" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -19887,8 +20652,11 @@
           <t>TOB</t>
         </is>
       </c>
-    </row>
-    <row r="145" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D144" s="3">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="145" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A145" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -19904,8 +20672,11 @@
           <t>WRT</t>
         </is>
       </c>
-    </row>
-    <row r="146" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D145" s="3">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="146" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A146" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -19921,8 +20692,11 @@
           <t>WBK</t>
         </is>
       </c>
-    </row>
-    <row r="147" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D146" s="3">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="147" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A147" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -19938,8 +20712,11 @@
           <t>WIL</t>
         </is>
       </c>
-    </row>
-    <row r="148" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D147" s="3">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="148" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A148" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -19955,8 +20732,11 @@
           <t>WNM</t>
         </is>
       </c>
-    </row>
-    <row r="149" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D148" s="3">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="149" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A149" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -19972,8 +20752,11 @@
           <t>WOK</t>
         </is>
       </c>
-    </row>
-    <row r="150" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D149" s="3">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="150" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A150" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -19989,8 +20772,11 @@
           <t>YOR</t>
         </is>
       </c>
-    </row>
-    <row r="151" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D150" s="3">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="151" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A151" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -20006,8 +20792,11 @@
           <t>LND</t>
         </is>
       </c>
-    </row>
-    <row r="152" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D151" s="3">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="152" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A152" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -20023,8 +20812,11 @@
           <t>ANT</t>
         </is>
       </c>
-    </row>
-    <row r="153" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D152" s="3">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="153" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A153" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -20040,8 +20832,11 @@
           <t>ARD</t>
         </is>
       </c>
-    </row>
-    <row r="154" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D153" s="3">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="154" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A154" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -20057,8 +20852,11 @@
           <t>ARM</t>
         </is>
       </c>
-    </row>
-    <row r="155" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D154" s="3">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="155" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A155" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -20074,8 +20872,11 @@
           <t>BLA</t>
         </is>
       </c>
-    </row>
-    <row r="156" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D155" s="3">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="156" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A156" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -20091,8 +20892,11 @@
           <t>BLY</t>
         </is>
       </c>
-    </row>
-    <row r="157" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D156" s="3">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="157" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A157" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -20108,8 +20912,11 @@
           <t>BNB</t>
         </is>
       </c>
-    </row>
-    <row r="158" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D157" s="3">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="158" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A158" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -20125,8 +20932,11 @@
           <t>BFS</t>
         </is>
       </c>
-    </row>
-    <row r="159" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D158" s="3">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="159" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A159" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -20142,8 +20952,11 @@
           <t>CKF</t>
         </is>
       </c>
-    </row>
-    <row r="160" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D159" s="3">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="160" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A160" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -20159,8 +20972,11 @@
           <t>CSR</t>
         </is>
       </c>
-    </row>
-    <row r="161" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D160" s="3">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="161" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A161" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -20176,8 +20992,11 @@
           <t>CLR</t>
         </is>
       </c>
-    </row>
-    <row r="162" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D161" s="3">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="162" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A162" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -20193,8 +21012,11 @@
           <t>CKT</t>
         </is>
       </c>
-    </row>
-    <row r="163" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D162" s="3">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="163" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A163" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -20210,8 +21032,11 @@
           <t>CGV</t>
         </is>
       </c>
-    </row>
-    <row r="164" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D163" s="3">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="164" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A164" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -20227,8 +21052,11 @@
           <t>DRY</t>
         </is>
       </c>
-    </row>
-    <row r="165" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D164" s="3">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="165" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A165" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -20244,8 +21072,11 @@
           <t>DOW</t>
         </is>
       </c>
-    </row>
-    <row r="166" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D165" s="3">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="166" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A166" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -20261,8 +21092,11 @@
           <t>DGN</t>
         </is>
       </c>
-    </row>
-    <row r="167" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D166" s="3">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="167" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A167" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -20278,8 +21112,11 @@
           <t>FER</t>
         </is>
       </c>
-    </row>
-    <row r="168" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D167" s="3">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="168" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A168" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -20295,8 +21132,11 @@
           <t>LRN</t>
         </is>
       </c>
-    </row>
-    <row r="169" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D168" s="3">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="169" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A169" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -20312,8 +21152,11 @@
           <t>LMV</t>
         </is>
       </c>
-    </row>
-    <row r="170" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D169" s="3">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="170" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A170" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -20329,8 +21172,11 @@
           <t>LSB</t>
         </is>
       </c>
-    </row>
-    <row r="171" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D170" s="3">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="171" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A171" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -20346,8 +21192,11 @@
           <t>MFT</t>
         </is>
       </c>
-    </row>
-    <row r="172" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D171" s="3">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="172" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A172" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -20363,8 +21212,11 @@
           <t>MYL</t>
         </is>
       </c>
-    </row>
-    <row r="173" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D172" s="3">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="173" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A173" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -20380,8 +21232,11 @@
           <t>NYM</t>
         </is>
       </c>
-    </row>
-    <row r="174" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D173" s="3">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="174" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A174" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -20397,8 +21252,11 @@
           <t>NTA</t>
         </is>
       </c>
-    </row>
-    <row r="175" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D174" s="3">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="175" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A175" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -20414,8 +21272,11 @@
           <t>NDN</t>
         </is>
       </c>
-    </row>
-    <row r="176" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D175" s="3">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="176" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A176" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -20431,8 +21292,11 @@
           <t>OMH</t>
         </is>
       </c>
-    </row>
-    <row r="177" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D176" s="3">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="177" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A177" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -20448,8 +21312,11 @@
           <t>STB</t>
         </is>
       </c>
-    </row>
-    <row r="178" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D177" s="3">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="178" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A178" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -20465,8 +21332,11 @@
           <t>ABE</t>
         </is>
       </c>
-    </row>
-    <row r="179" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D178" s="3">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="179" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A179" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -20482,8 +21352,11 @@
           <t>ABD</t>
         </is>
       </c>
-    </row>
-    <row r="180" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D179" s="3">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="180" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A180" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -20499,8 +21372,11 @@
           <t>ANS</t>
         </is>
       </c>
-    </row>
-    <row r="181" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D180" s="3">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="181" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A181" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -20516,8 +21392,11 @@
           <t>AGB</t>
         </is>
       </c>
-    </row>
-    <row r="182" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D181" s="3">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="182" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A182" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -20533,8 +21412,11 @@
           <t>CLK</t>
         </is>
       </c>
-    </row>
-    <row r="183" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D182" s="3">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="183" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A183" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -20550,8 +21432,11 @@
           <t>DGY</t>
         </is>
       </c>
-    </row>
-    <row r="184" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D183" s="3">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="184" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A184" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -20567,8 +21452,11 @@
           <t>DND</t>
         </is>
       </c>
-    </row>
-    <row r="185" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D184" s="3">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="185" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A185" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -20584,8 +21472,11 @@
           <t>EAY</t>
         </is>
       </c>
-    </row>
-    <row r="186" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D185" s="3">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="186" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A186" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -20601,8 +21492,11 @@
           <t>EDU</t>
         </is>
       </c>
-    </row>
-    <row r="187" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D186" s="3">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="187" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A187" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -20618,8 +21512,11 @@
           <t>ELN</t>
         </is>
       </c>
-    </row>
-    <row r="188" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D187" s="3">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="188" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A188" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -20635,8 +21532,11 @@
           <t>ERW</t>
         </is>
       </c>
-    </row>
-    <row r="189" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D188" s="3">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="189" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A189" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -20652,8 +21552,11 @@
           <t>EDH</t>
         </is>
       </c>
-    </row>
-    <row r="190" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D189" s="3">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="190" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A190" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -20669,8 +21572,11 @@
           <t>ELS</t>
         </is>
       </c>
-    </row>
-    <row r="191" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D190" s="3">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="191" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A191" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -20686,8 +21592,11 @@
           <t>FAL</t>
         </is>
       </c>
-    </row>
-    <row r="192" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D191" s="3">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="192" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A192" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -20703,8 +21612,11 @@
           <t>FIF</t>
         </is>
       </c>
-    </row>
-    <row r="193" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D192" s="3">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="193" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A193" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -20720,8 +21632,11 @@
           <t>GLG</t>
         </is>
       </c>
-    </row>
-    <row r="194" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D193" s="3">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="194" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A194" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -20737,8 +21652,11 @@
           <t>HLD</t>
         </is>
       </c>
-    </row>
-    <row r="195" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D194" s="3">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="195" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A195" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -20754,8 +21672,11 @@
           <t>IVC</t>
         </is>
       </c>
-    </row>
-    <row r="196" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D195" s="3">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="196" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A196" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -20771,8 +21692,11 @@
           <t>MLN</t>
         </is>
       </c>
-    </row>
-    <row r="197" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D196" s="3">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="197" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A197" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -20788,8 +21712,11 @@
           <t>MRY</t>
         </is>
       </c>
-    </row>
-    <row r="198" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D197" s="3">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="198" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A198" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -20805,8 +21732,11 @@
           <t>NAY</t>
         </is>
       </c>
-    </row>
-    <row r="199" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D198" s="3">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="199" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A199" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -20822,8 +21752,11 @@
           <t>NLK</t>
         </is>
       </c>
-    </row>
-    <row r="200" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D199" s="3">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="200" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A200" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -20839,8 +21772,11 @@
           <t>ORK</t>
         </is>
       </c>
-    </row>
-    <row r="201" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D200" s="3">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="201" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A201" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -20856,8 +21792,11 @@
           <t>PKN</t>
         </is>
       </c>
-    </row>
-    <row r="202" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D201" s="3">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="202" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A202" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -20873,8 +21812,11 @@
           <t>RFW</t>
         </is>
       </c>
-    </row>
-    <row r="203" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D202" s="3">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="203" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A203" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -20890,8 +21832,11 @@
           <t>SCB</t>
         </is>
       </c>
-    </row>
-    <row r="204" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D203" s="3">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="204" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A204" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -20907,8 +21852,11 @@
           <t>ZET</t>
         </is>
       </c>
-    </row>
-    <row r="205" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D204" s="3">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="205" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A205" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -20924,8 +21872,11 @@
           <t>SAY</t>
         </is>
       </c>
-    </row>
-    <row r="206" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D205" s="3">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="206" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A206" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -20941,8 +21892,11 @@
           <t>SLK</t>
         </is>
       </c>
-    </row>
-    <row r="207" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D206" s="3">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="207" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A207" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -20958,8 +21912,11 @@
           <t>STG</t>
         </is>
       </c>
-    </row>
-    <row r="208" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D207" s="3">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="208" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A208" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -20975,8 +21932,11 @@
           <t>WDU</t>
         </is>
       </c>
-    </row>
-    <row r="209" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D208" s="3">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="209" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A209" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -20992,8 +21952,11 @@
           <t>WLN</t>
         </is>
       </c>
-    </row>
-    <row r="210" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D209" s="3">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="210" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A210" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -21009,8 +21972,11 @@
           <t>BGW</t>
         </is>
       </c>
-    </row>
-    <row r="211" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D210" s="3">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="211" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A211" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -21026,8 +21992,11 @@
           <t>BGE</t>
         </is>
       </c>
-    </row>
-    <row r="212" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D211" s="3">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="212" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A212" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -21043,8 +22012,11 @@
           <t>CRF</t>
         </is>
       </c>
-    </row>
-    <row r="213" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D212" s="3">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="213" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A213" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -21060,8 +22032,11 @@
           <t>CMN</t>
         </is>
       </c>
-    </row>
-    <row r="214" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D213" s="3">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="214" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A214" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -21077,8 +22052,11 @@
           <t>CGN</t>
         </is>
       </c>
-    </row>
-    <row r="215" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D214" s="3">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="215" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A215" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -21094,8 +22072,11 @@
           <t>DEN</t>
         </is>
       </c>
-    </row>
-    <row r="216" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D215" s="3">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="216" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A216" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -21111,8 +22092,11 @@
           <t>FLN</t>
         </is>
       </c>
-    </row>
-    <row r="217" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D216" s="3">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="217" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A217" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -21128,8 +22112,11 @@
           <t>GWN</t>
         </is>
       </c>
-    </row>
-    <row r="218" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D217" s="3">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="218" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A218" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -21145,8 +22132,11 @@
           <t>AGY</t>
         </is>
       </c>
-    </row>
-    <row r="219" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D218" s="3">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="219" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A219" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -21162,8 +22152,11 @@
           <t>MTY</t>
         </is>
       </c>
-    </row>
-    <row r="220" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D219" s="3">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="220" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A220" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -21175,8 +22168,11 @@
           <t>MDW</t>
         </is>
       </c>
-    </row>
-    <row r="221" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D220" s="3">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="221" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A221" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -21188,8 +22184,11 @@
           <t>CAY</t>
         </is>
       </c>
-    </row>
-    <row r="222" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D221" s="3">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="222" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A222" s="3" t="inlineStr">
         <is>
           <t>United Kingdom</t>
@@ -21200,6 +22199,9 @@
         <is>
           <t>CWY</t>
         </is>
+      </c>
+      <c r="D222" s="3">
+        <v>221</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Germany SAP T005S state mapping
</commit_message>
<xml_diff>
--- a/doc/state_mapping.xlsx
+++ b/doc/state_mapping.xlsx
@@ -16,6 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="France T005S Map" sheetId="2" r:id="rId2"/>
     <sheet name="GB T005S Map" sheetId="3" r:id="rId6"/>
+    <sheet name="Germany T005S Map" sheetId="4" r:id="rId7"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
@@ -22207,4 +22208,355 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:D17"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="3" width="17" customWidth="1"/>
+    <col min="4" max="4" width="10" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="2" t="s">
+        <v>343</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>344</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>345</v>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>SH</t>
+        </is>
+      </c>
+      <c r="D2" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>HH</t>
+        </is>
+      </c>
+      <c r="D3" s="3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>03</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>NI</t>
+        </is>
+      </c>
+      <c r="D4" s="3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>04</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>HB</t>
+        </is>
+      </c>
+      <c r="D5" s="3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>05</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>NW</t>
+        </is>
+      </c>
+      <c r="D6" s="3">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>06</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>HE</t>
+        </is>
+      </c>
+      <c r="D7" s="3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>07</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>RP</t>
+        </is>
+      </c>
+      <c r="D8" s="3">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>BW</t>
+        </is>
+      </c>
+      <c r="D9" s="3">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>09</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>BY</t>
+        </is>
+      </c>
+      <c r="D10" s="3">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>SL</t>
+        </is>
+      </c>
+      <c r="D11" s="3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="D12" s="3">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="D13" s="3">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>MV</t>
+        </is>
+      </c>
+      <c r="D14" s="3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>SN</t>
+        </is>
+      </c>
+      <c r="D15" s="3">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="D16" s="3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>TH</t>
+        </is>
+      </c>
+      <c r="D17" s="3">
+        <v>16</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
docs: add Netherlands province mapping tab
</commit_message>
<xml_diff>
--- a/doc/state_mapping.xlsx
+++ b/doc/state_mapping.xlsx
@@ -20,6 +20,7 @@
     <sheet name="Austria T005S Map" sheetId="5" r:id="rId5"/>
     <sheet name="China T005S Map" sheetId="6" r:id="rId6"/>
     <sheet name="Spain T005S Map" sheetId="7" r:id="rId10"/>
+    <sheet name="Netherlands T005S Map" sheetId="8" r:id="rId11"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
@@ -22976,4 +22977,177 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="18" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="17" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="17" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="10" hidden="0" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="2" t="str">
+        <v>Country</v>
+      </c>
+      <c r="B1" s="2" t="str">
+        <v>SAP Value</v>
+      </c>
+      <c r="C1" s="2" t="str">
+        <v>EC Value</v>
+      </c>
+      <c r="D1" s="2" t="str">
+        <v>No.</v>
+      </c>
+    </row>
+    <row r="2" ht="19" customHeight="1">
+      <c r="A2" s="3" t="str">
+        <v>Netherlands</v>
+      </c>
+      <c r="B2" s="5"/>
+      <c r="C2" s="4" t="str">
+        <v>DR</v>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" ht="19" customHeight="1">
+      <c r="A3" s="3" t="str">
+        <v>Netherlands</v>
+      </c>
+      <c r="B3" s="5"/>
+      <c r="C3" s="4" t="str">
+        <v>FL</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" ht="19" customHeight="1">
+      <c r="A4" s="3" t="str">
+        <v>Netherlands</v>
+      </c>
+      <c r="B4" s="5"/>
+      <c r="C4" s="4" t="str">
+        <v>FR</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" ht="19" customHeight="1">
+      <c r="A5" s="3" t="str">
+        <v>Netherlands</v>
+      </c>
+      <c r="B5" s="5"/>
+      <c r="C5" s="4" t="str">
+        <v>GE</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" ht="19" customHeight="1">
+      <c r="A6" s="3" t="str">
+        <v>Netherlands</v>
+      </c>
+      <c r="B6" s="5"/>
+      <c r="C6" s="4" t="str">
+        <v>GR</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" ht="19" customHeight="1">
+      <c r="A7" s="3" t="str">
+        <v>Netherlands</v>
+      </c>
+      <c r="B7" s="5"/>
+      <c r="C7" s="4" t="str">
+        <v>LI</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" ht="19" customHeight="1">
+      <c r="A8" s="3" t="str">
+        <v>Netherlands</v>
+      </c>
+      <c r="B8" s="5"/>
+      <c r="C8" s="4" t="str">
+        <v>NB</v>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" ht="19" customHeight="1">
+      <c r="A9" s="3" t="str">
+        <v>Netherlands</v>
+      </c>
+      <c r="B9" s="5"/>
+      <c r="C9" s="4" t="str">
+        <v>NH</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" ht="19" customHeight="1">
+      <c r="A10" s="3" t="str">
+        <v>Netherlands</v>
+      </c>
+      <c r="B10" s="5"/>
+      <c r="C10" s="4" t="str">
+        <v>OV</v>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" ht="19" customHeight="1">
+      <c r="A11" s="3" t="str">
+        <v>Netherlands</v>
+      </c>
+      <c r="B11" s="5"/>
+      <c r="C11" s="4" t="str">
+        <v>ZH</v>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" ht="19" customHeight="1">
+      <c r="A12" s="3" t="str">
+        <v>Netherlands</v>
+      </c>
+      <c r="B12" s="5"/>
+      <c r="C12" s="4" t="str">
+        <v>UT</v>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" ht="19" customHeight="1">
+      <c r="A13" s="3" t="str">
+        <v>Netherlands</v>
+      </c>
+      <c r="B13" s="5"/>
+      <c r="C13" s="4" t="str">
+        <v>ZE</v>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>12</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>